<commit_message>
feat: add certificate gallery view, candidate stepper, single PDF download, and session persistence
</commit_message>
<xml_diff>
--- a/IIMcandidatelist.xlsx
+++ b/IIMcandidatelist.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\anmol\OneDrive\Documents\OneDrive\Documents\anmolrkumar\certs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FAD09EFD-4733-4F85-A86C-99DF312D3210}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17D2D1B7-B8C7-4144-94D6-C4FDF9AF8BD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15270" xr2:uid="{1A645ADA-15BB-41E2-B9A0-7FEF42D44569}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="22">
   <si>
     <t>Roll Number</t>
   </si>
@@ -94,6 +94,12 @@
   </si>
   <si>
     <t>xyz@gmail.com</t>
+  </si>
+  <si>
+    <t>xyz1@gmail.com</t>
+  </si>
+  <si>
+    <t>abc@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -620,7 +626,7 @@
         <v>14</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
@@ -634,7 +640,7 @@
         <v>17</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>